<commit_message>
update 2026-09-27 22:45 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/57cfe36beb_Financial_Analysis_2026.xlsx
+++ b/57cfe36beb_Financial_Analysis_2026.xlsx
@@ -6626,13 +6626,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>38500</v>
+        <v>30500</v>
       </c>
       <c r="D4" t="n">
-        <v>39.5</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="5">
@@ -6648,7 +6648,7 @@
         <v>20477.9</v>
       </c>
       <c r="D5" t="n">
-        <v>21</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="6">
@@ -6658,13 +6658,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>14020</v>
+        <v>13020</v>
       </c>
       <c r="D6" t="n">
-        <v>14.4</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="7">
@@ -6680,7 +6680,7 @@
         <v>8470.620000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>8.699999999999999</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="8">
@@ -6696,7 +6696,7 @@
         <v>5750.549999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="9">
@@ -6712,7 +6712,7 @@
         <v>3199.98</v>
       </c>
       <c r="D9" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="10">
@@ -6728,7 +6728,7 @@
         <v>1766</v>
       </c>
       <c r="D10" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -6744,7 +6744,7 @@
         <v>1670.4</v>
       </c>
       <c r="D11" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="12">
@@ -6760,7 +6760,7 @@
         <v>1419.4</v>
       </c>
       <c r="D12" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="13">
@@ -6776,7 +6776,7 @@
         <v>1192</v>
       </c>
       <c r="D13" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="14">
@@ -6871,11 +6871,11 @@
         <v>1</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>46085</v>
+        <v>46090</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NBE ATM713</t>
+          <t>NBE ATM666</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>8000</v>
+        <v>3300</v>
       </c>
     </row>
     <row r="5">
@@ -6892,11 +6892,11 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>46090</v>
+        <v>46085</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NBE ATM666</t>
+          <t>NBE ATM713</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -6905,7 +6905,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>3300</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="6">
@@ -6913,11 +6913,11 @@
         <v>3</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>46085</v>
+        <v>46174</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NBE ATM713</t>
+          <t>NBE ATM714</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -6934,7 +6934,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>46174</v>
+        <v>46184</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -6955,20 +6955,20 @@
         <v>5</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>46184</v>
+        <v>46116</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NBE ATM714</t>
+          <t>AMAZON Cai</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>تسوق أونلاين</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>3000</v>
+        <v>2385.99</v>
       </c>
     </row>
     <row r="9">
@@ -6976,20 +6976,20 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>46116</v>
+        <v>46056</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMAZON Cai</t>
+          <t>FAWRY*RUMBLE BYM store</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>تسوق أونلاين</t>
+          <t>مدفوعات وتحويلات</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>2385.99</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="10">
@@ -6997,11 +6997,11 @@
         <v>7</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>46056</v>
+        <v>46058</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FAWRY*RUMBLE BYM store</t>
+          <t>QNBS-0082 GIZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -7018,16 +7018,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="9" t="n">
-        <v>46058</v>
+        <v>46132</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>QNBS-0082 GIZ</t>
+          <t>BM EL MARYOTYA BR 1 G</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>مدفوعات وتحويلات</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
@@ -7039,16 +7039,16 @@
         <v>9</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>46132</v>
+        <v>46210</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BM EL MARYOTYA BR 1 G</t>
+          <t>NBE ATM713</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
@@ -7060,16 +7060,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>46210</v>
+        <v>46270</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NBE ATM713</t>
+          <t>BDC ELHARAM C</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
@@ -7081,11 +7081,11 @@
         <v>11</v>
       </c>
       <c r="B14" s="9" t="n">
-        <v>46270</v>
+        <v>46157</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BDC ELHARAM C</t>
+          <t>AL NASSER GI</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -7094,7 +7094,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2000</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="15">
@@ -7102,11 +7102,11 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="n">
-        <v>46157</v>
+        <v>46159</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AL NASSER GI</t>
+          <t>Flash Technologies Cai</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -7115,7 +7115,7 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1985</v>
+        <v>1887.9</v>
       </c>
     </row>
     <row r="16">
@@ -7123,11 +7123,11 @@
         <v>13</v>
       </c>
       <c r="B16" s="9" t="n">
-        <v>46159</v>
+        <v>46052</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Flash Technologies Cai</t>
+          <t>85 HARAM ST GIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -7136,7 +7136,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1887.9</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="17">
@@ -7144,16 +7144,16 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="n">
-        <v>46052</v>
+        <v>46115</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>85 HARAM ST GIZ</t>
+          <t>NBK-EGYPT MINA_PALACE 15</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>مدفوعات وتحويلات</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
@@ -7165,16 +7165,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="9" t="n">
-        <v>46115</v>
+        <v>46246</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NBK-EGYPT MINA_PALACE 15</t>
+          <t>BM HUB OLA DEBOMAT 2TH C</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>مدفوعات وتحويلات</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
@@ -7186,11 +7186,11 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="n">
-        <v>46246</v>
+        <v>46182</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BM HUB OLA DEBOMAT 2TH C</t>
+          <t>KASHIER*AboSh Cai</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -7199,7 +7199,7 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1500</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="20">
@@ -7207,20 +7207,20 @@
         <v>17</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>46182</v>
+        <v>46235</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KASHIER*AboSh Cai</t>
+          <t>U TURN GI</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1350</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="21">
@@ -7228,20 +7228,20 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>46235</v>
+        <v>46156</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>U TURN GI</t>
+          <t>EL EZABY HEL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>أخرى (غير مصنف)</t>
+          <t>صحة وصيدليات</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1150</v>
+        <v>1109.4</v>
       </c>
     </row>
     <row r="22">
@@ -7249,20 +7249,20 @@
         <v>19</v>
       </c>
       <c r="B22" s="9" t="n">
-        <v>46156</v>
+        <v>46266</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EL EZABY HEL</t>
+          <t>BDC HARAM H</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>صحة وصيدليات</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1109.4</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="23">
@@ -7270,20 +7270,20 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>46266</v>
+        <v>46055</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BDC HARAM H</t>
+          <t>NBE ATM714</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -7604,7 +7604,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>38500</v>
+        <v>30500</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -7619,7 +7619,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>49886.53</v>
+        <v>57886.53</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update 2026-09-28 00:08 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/57cfe36beb_Financial_Analysis_2026.xlsx
+++ b/57cfe36beb_Financial_Analysis_2026.xlsx
@@ -37,7 +37,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="000E2A47"/>
       <sz val="14"/>
     </font>
     <font>
@@ -55,11 +55,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="000E2A47"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E7D32"/>
+      <color rgb="0015803D"/>
     </font>
   </fonts>
   <fills count="3">
@@ -71,7 +71,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="000E2A47"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
update 2026-10-01 19:43 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/57cfe36beb_Financial_Analysis_2026.xlsx
+++ b/57cfe36beb_Financial_Analysis_2026.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G202"/>
+  <dimension ref="A1:G211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>كشف معاملات البطاقة 3390 (28/01/2026 - 19/09/2026)</t>
+          <t>كشف معاملات البطاقة 3390 (28/01/2026 - 01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -6251,6 +6251,261 @@
       </c>
       <c r="G202" s="5" t="n">
         <v>4602.41</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>يوسف نبيل نصيف رزق</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F203" s="5" t="n"/>
+      <c r="G203" s="5" t="n">
+        <v>6602.41</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C204" s="4" t="inlineStr">
+        <is>
+          <t>CIB-FAWRY PLUS FAISAL G</t>
+        </is>
+      </c>
+      <c r="D204" s="4" t="inlineStr">
+        <is>
+          <t>مدفوعات وتحويلات</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F204" s="5" t="n">
+        <v>995.79</v>
+      </c>
+      <c r="G204" s="5" t="n">
+        <v>5602.41</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C205" s="4" t="inlineStr">
+        <is>
+          <t>FAWRY*DOCTOR BIKE AU</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr">
+        <is>
+          <t>مدفوعات وتحويلات</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="F205" s="5" t="n">
+        <v>495.79</v>
+      </c>
+      <c r="G205" s="5" t="n">
+        <v>5102.41</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
+        <is>
+          <t>Vodafone Top Up APP Sma</t>
+        </is>
+      </c>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>موبايل وإنترنت</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="F206" s="5" t="n">
+        <v>352.79</v>
+      </c>
+      <c r="G206" s="5" t="n">
+        <v>4959.41</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>CHILL OUT DAR ELSALAM</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>كافيهات وترفيه</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="n">
+        <v>226</v>
+      </c>
+      <c r="F207" s="5" t="n">
+        <v>126.79</v>
+      </c>
+      <c r="G207" s="5" t="n">
+        <v>4733.41</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>Vodafone Top Up APP Sma</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>موبايل وإنترنت</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="n">
+        <v>126</v>
+      </c>
+      <c r="F208" s="5" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G208" s="5" t="n">
+        <v>4607.41</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>ESSAM MOHAMED TAHA MAHROUS IBRAHIM</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="F209" s="5" t="n"/>
+      <c r="G209" s="5" t="n">
+        <v>5087.41</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>يوسف نبيل نصيف رزق</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F210" s="5" t="n"/>
+      <c r="G210" s="5" t="n">
+        <v>22087.41</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>BDC ELSTODYOHAT ALANTA 6</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>مشتريات ومحلات</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F211" s="5" t="n">
+        <v>15475.79</v>
+      </c>
+      <c r="G211" s="5" t="n">
+        <v>20087.41</v>
       </c>
     </row>
   </sheetData>
@@ -6264,7 +6519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6527,47 +6782,72 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>8617.27</v>
+        <v>10612.27</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>8617.27</v>
+        <v>10612.27</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>8570</v>
+        <v>11050</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-47.27000000000044</v>
+        <v>437.7299999999996</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>17000</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>199</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>97386.53</v>
-      </c>
-      <c r="D13" s="8" t="n">
+      <c r="B14" s="7" t="n">
+        <v>208</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>101381.53</v>
+      </c>
+      <c r="D14" s="8" t="n">
         <v>9000</v>
       </c>
-      <c r="E13" s="8" t="n">
-        <v>88386.53</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>92245</v>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>3858.470000000001</v>
+      <c r="E14" s="8" t="n">
+        <v>92381.53</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>111725</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>19343.47</v>
       </c>
     </row>
   </sheetData>
@@ -6632,7 +6912,7 @@
         <v>30500</v>
       </c>
       <c r="D4" t="n">
-        <v>34.5</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -6642,13 +6922,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>20477.9</v>
+        <v>22477.9</v>
       </c>
       <c r="D5" t="n">
-        <v>23.2</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="6">
@@ -6658,13 +6938,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>13020</v>
+        <v>14520</v>
       </c>
       <c r="D6" t="n">
-        <v>14.7</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="7">
@@ -6674,13 +6954,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>8470.620000000001</v>
+        <v>8739.620000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="8">
@@ -6696,7 +6976,7 @@
         <v>5750.549999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="9">
@@ -6712,7 +6992,7 @@
         <v>3199.98</v>
       </c>
       <c r="D9" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10">
@@ -6728,7 +7008,7 @@
         <v>1766</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="11">
@@ -6744,7 +7024,7 @@
         <v>1670.4</v>
       </c>
       <c r="D11" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="12">
@@ -6760,7 +7040,7 @@
         <v>1419.4</v>
       </c>
       <c r="D12" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="13">
@@ -6786,13 +7066,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>571</v>
+        <v>797</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15">
@@ -7081,11 +7361,11 @@
         <v>11</v>
       </c>
       <c r="B14" s="9" t="n">
-        <v>46157</v>
+        <v>46296</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AL NASSER GI</t>
+          <t>BDC ELSTODYOHAT ALANTA 6</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -7094,7 +7374,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1985</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="15">
@@ -7102,11 +7382,11 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="n">
-        <v>46159</v>
+        <v>46157</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Flash Technologies Cai</t>
+          <t>AL NASSER GI</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -7115,7 +7395,7 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1887.9</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="16">
@@ -7123,11 +7403,11 @@
         <v>13</v>
       </c>
       <c r="B16" s="9" t="n">
-        <v>46052</v>
+        <v>46159</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>85 HARAM ST GIZ</t>
+          <t>Flash Technologies Cai</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -7136,7 +7416,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1500</v>
+        <v>1887.9</v>
       </c>
     </row>
     <row r="17">
@@ -7144,16 +7424,16 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="n">
-        <v>46115</v>
+        <v>46052</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NBK-EGYPT MINA_PALACE 15</t>
+          <t>85 HARAM ST GIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>مدفوعات وتحويلات</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
@@ -7165,16 +7445,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="9" t="n">
-        <v>46246</v>
+        <v>46115</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BM HUB OLA DEBOMAT 2TH C</t>
+          <t>NBK-EGYPT MINA_PALACE 15</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>مدفوعات وتحويلات</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
@@ -7186,11 +7466,11 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="n">
-        <v>46182</v>
+        <v>46246</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KASHIER*AboSh Cai</t>
+          <t>BM HUB OLA DEBOMAT 2TH C</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -7199,7 +7479,7 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1350</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="20">
@@ -7207,20 +7487,20 @@
         <v>17</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>46235</v>
+        <v>46182</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>U TURN GI</t>
+          <t>KASHIER*AboSh Cai</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>أخرى (غير مصنف)</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1150</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="21">
@@ -7228,20 +7508,20 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>46156</v>
+        <v>46235</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EL EZABY HEL</t>
+          <t>U TURN GI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>صحة وصيدليات</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1109.4</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="22">
@@ -7249,20 +7529,20 @@
         <v>19</v>
       </c>
       <c r="B22" s="9" t="n">
-        <v>46266</v>
+        <v>46156</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BDC HARAM H</t>
+          <t>EL EZABY HEL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>صحة وصيدليات</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1100</v>
+        <v>1109.4</v>
       </c>
     </row>
     <row r="23">
@@ -7270,20 +7550,20 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>46055</v>
+        <v>46266</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NBE ATM714</t>
+          <t>BDC HARAM H</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
     </row>
   </sheetData>
@@ -7336,10 +7616,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>89000</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="5">
@@ -7349,10 +7629,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>960</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="6">
@@ -7466,7 +7746,7 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>92245</v>
+        <v>111725</v>
       </c>
     </row>
   </sheetData>
@@ -7491,7 +7771,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>مؤشرات عامة - فترة 28/01/2026 حتى 19/09/2026</t>
+          <t>مؤشرات عامة - فترة 28/01/2026 حتى 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -7519,7 +7799,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
@@ -7530,7 +7810,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
@@ -7541,7 +7821,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -7571,7 +7851,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>97386.53</v>
+        <v>101381.53</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -7593,7 +7873,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>88386.53</v>
+        <v>92381.53</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
@@ -7619,7 +7899,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>57886.53</v>
+        <v>61881.53</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
@@ -7630,7 +7910,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>92245</v>
+        <v>111725</v>
       </c>
       <c r="C13" t="inlineStr"/>
     </row>
@@ -7641,7 +7921,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>3858.47</v>
+        <v>19343.47</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
@@ -7652,7 +7932,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>376.11</v>
+        <v>374.01</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
@@ -7663,7 +7943,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>11448.88</v>
+        <v>11385</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
@@ -7685,7 +7965,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>4602.41</v>
+        <v>20087.41</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
@@ -7696,7 +7976,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.79</v>
+        <v>15475.79</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
@@ -7707,7 +7987,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>4601.62</v>
+        <v>4611.62</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -7726,7 +8006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11361,6 +11641,132 @@
         <v>4601.62</v>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>CIB-FAWRY PLUS FAISAL G</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>5602.41</v>
+      </c>
+      <c r="D175" t="n">
+        <v>995.79</v>
+      </c>
+      <c r="E175" t="n">
+        <v>4606.62</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>FAWRY*DOCTOR BIKE AU</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>5102.41</v>
+      </c>
+      <c r="D176" t="n">
+        <v>495.79</v>
+      </c>
+      <c r="E176" t="n">
+        <v>4606.62</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Vodafone Top Up APP Sma</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>4959.41</v>
+      </c>
+      <c r="D177" t="n">
+        <v>352.79</v>
+      </c>
+      <c r="E177" t="n">
+        <v>4606.62</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CHILL OUT DAR ELSALAM</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>4733.41</v>
+      </c>
+      <c r="D178" t="n">
+        <v>126.79</v>
+      </c>
+      <c r="E178" t="n">
+        <v>4606.62</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Vodafone Top Up APP Sma</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>4607.41</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E179" t="n">
+        <v>4606.62</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>BDC ELSTODYOHAT ALANTA 6</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>20087.41</v>
+      </c>
+      <c r="D180" t="n">
+        <v>15475.79</v>
+      </c>
+      <c r="E180" t="n">
+        <v>4611.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update 2026-10-01 22:26 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/57cfe36beb_Financial_Analysis_2026.xlsx
+++ b/57cfe36beb_Financial_Analysis_2026.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G211"/>
+  <dimension ref="A1:G213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E145" s="5" t="n">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E147" s="5" t="n">
@@ -5637,7 +5637,7 @@
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E181" s="5" t="n">
@@ -5724,7 +5724,7 @@
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E184" s="5" t="n">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E186" s="5" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E187" s="5" t="n">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E188" s="5" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E193" s="5" t="n">
@@ -6255,29 +6255,29 @@
     </row>
     <row r="203">
       <c r="A203" s="3" t="n">
-        <v>46291</v>
+        <v>46287</v>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>مصروف</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>يوسف نبيل نصيف رزق</t>
+          <t>CHOCO STORE</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>بقالة وسوبر ماركت</t>
         </is>
       </c>
       <c r="E203" s="5" t="n">
-        <v>2000</v>
+        <v>5</v>
       </c>
       <c r="F203" s="5" t="n"/>
       <c r="G203" s="5" t="n">
-        <v>6602.41</v>
+        <v>4597.41</v>
       </c>
     </row>
     <row r="204">
@@ -6286,27 +6286,25 @@
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>مصروف</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>CIB-FAWRY PLUS FAISAL G</t>
+          <t>يوسف نبيل نصيف رزق</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>مدفوعات وتحويلات</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="E204" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F204" s="5" t="n">
-        <v>995.79</v>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="F204" s="5" t="n"/>
       <c r="G204" s="5" t="n">
-        <v>5602.41</v>
+        <v>6597.41</v>
       </c>
     </row>
     <row r="205">
@@ -6320,7 +6318,7 @@
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>FAWRY*DOCTOR BIKE AU</t>
+          <t>CIB-FAWRY PLUS FAISAL G</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -6329,18 +6327,18 @@
         </is>
       </c>
       <c r="E205" s="5" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F205" s="5" t="n">
-        <v>495.79</v>
+        <v>995.79</v>
       </c>
       <c r="G205" s="5" t="n">
-        <v>5102.41</v>
+        <v>5597.41</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
@@ -6349,22 +6347,22 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Vodafone Top Up APP Sma</t>
+          <t>FAWRY*DOCTOR BIKE AU</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>موبايل وإنترنت</t>
+          <t>مدفوعات وتحويلات</t>
         </is>
       </c>
       <c r="E206" s="5" t="n">
-        <v>143</v>
+        <v>500</v>
       </c>
       <c r="F206" s="5" t="n">
-        <v>352.79</v>
+        <v>495.79</v>
       </c>
       <c r="G206" s="5" t="n">
-        <v>4959.41</v>
+        <v>5097.41</v>
       </c>
     </row>
     <row r="207">
@@ -6378,22 +6376,22 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>CHILL OUT DAR ELSALAM</t>
+          <t>Vodafone Top Up APP Sma</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>كافيهات وترفيه</t>
+          <t>موبايل وإنترنت</t>
         </is>
       </c>
       <c r="E207" s="5" t="n">
-        <v>226</v>
+        <v>143</v>
       </c>
       <c r="F207" s="5" t="n">
-        <v>126.79</v>
+        <v>352.79</v>
       </c>
       <c r="G207" s="5" t="n">
-        <v>4733.41</v>
+        <v>4954.41</v>
       </c>
     </row>
     <row r="208">
@@ -6407,105 +6405,161 @@
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Vodafone Top Up APP Sma</t>
+          <t>CHILL OUT DAR ELSALAM</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>موبايل وإنترنت</t>
+          <t>كافيهات وترفيه</t>
         </is>
       </c>
       <c r="E208" s="5" t="n">
-        <v>126</v>
+        <v>226</v>
       </c>
       <c r="F208" s="5" t="n">
-        <v>0.79</v>
+        <v>126.79</v>
       </c>
       <c r="G208" s="5" t="n">
-        <v>4607.41</v>
+        <v>4728.41</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>مصروف</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>ESSAM MOHAMED TAHA MAHROUS IBRAHIM</t>
+          <t>Vodafone Top Up APP Sma</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>موبايل وإنترنت</t>
         </is>
       </c>
       <c r="E209" s="5" t="n">
-        <v>480</v>
-      </c>
-      <c r="F209" s="5" t="n"/>
+        <v>126</v>
+      </c>
+      <c r="F209" s="5" t="n">
+        <v>0.79</v>
+      </c>
       <c r="G209" s="5" t="n">
-        <v>5087.41</v>
+        <v>4602.41</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>مصروف</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>يوسف نبيل نصيف رزق</t>
+          <t>CHOCO STORE</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>بقالة وسوبر ماركت</t>
         </is>
       </c>
       <c r="E210" s="5" t="n">
-        <v>17000</v>
+        <v>5</v>
       </c>
       <c r="F210" s="5" t="n"/>
       <c r="G210" s="5" t="n">
-        <v>22087.41</v>
+        <v>4597.41</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>ESSAM MOHAMED TAHA MAHROUS IBRAHIM</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="F211" s="5" t="n"/>
+      <c r="G211" s="5" t="n">
+        <v>5077.41</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="n">
         <v>46296</v>
       </c>
-      <c r="B211" s="4" t="inlineStr">
-        <is>
-          <t>مصروف</t>
-        </is>
-      </c>
-      <c r="C211" s="4" t="inlineStr">
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>يوسف نبيل نصيف رزق</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>وارد</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F212" s="5" t="n"/>
+      <c r="G212" s="5" t="n">
+        <v>22077.41</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
         <is>
           <t>BDC ELSTODYOHAT ALANTA 6</t>
         </is>
       </c>
-      <c r="D211" s="4" t="inlineStr">
-        <is>
-          <t>مشتريات ومحلات</t>
-        </is>
-      </c>
-      <c r="E211" s="5" t="n">
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>سحب نقدي (ATM)</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="F211" s="5" t="n">
+      <c r="F213" s="5" t="n">
         <v>15475.79</v>
       </c>
-      <c r="G211" s="5" t="n">
-        <v>20087.41</v>
+      <c r="G213" s="5" t="n">
+        <v>20077.41</v>
       </c>
     </row>
   </sheetData>
@@ -6782,22 +6836,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>10612.27</v>
+        <v>10622.27</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>10612.27</v>
+        <v>10622.27</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>11050</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>437.7299999999996</v>
+        <v>427.7299999999996</v>
       </c>
     </row>
     <row r="13">
@@ -6832,22 +6886,22 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>101381.53</v>
+        <v>101391.53</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>9000</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>92381.53</v>
+        <v>92391.53</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111725</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>19343.47</v>
+        <v>19333.47</v>
       </c>
     </row>
   </sheetData>
@@ -6906,45 +6960,45 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>30500</v>
+        <v>39500</v>
       </c>
       <c r="D4" t="n">
-        <v>33</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>مدفوعات وتحويلات</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>22477.9</v>
+        <v>14520</v>
       </c>
       <c r="D5" t="n">
-        <v>24.3</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>مدفوعات وتحويلات</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>14520</v>
+        <v>13477.9</v>
       </c>
       <c r="D6" t="n">
-        <v>15.7</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="7">
@@ -7018,10 +7072,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1670.4</v>
+        <v>1680.4</v>
       </c>
       <c r="D11" t="n">
         <v>1.8</v>
@@ -7349,7 +7403,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
@@ -7370,7 +7424,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E14" s="6" t="n">
@@ -7559,7 +7613,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>سحب نقدي (ATM)</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
@@ -7810,7 +7864,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
@@ -7851,7 +7905,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>101381.53</v>
+        <v>101391.53</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -7873,7 +7927,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>92381.53</v>
+        <v>92391.53</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
@@ -7884,7 +7938,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>30500</v>
+        <v>39500</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -7899,7 +7953,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>61881.53</v>
+        <v>52891.53</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
@@ -7921,7 +7975,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>19343.47</v>
+        <v>19333.47</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
@@ -7932,7 +7986,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>374.01</v>
+        <v>374.05</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
@@ -7943,7 +7997,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>11385</v>
+        <v>11386.23</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
@@ -7965,7 +8019,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>20087.41</v>
+        <v>20077.41</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
@@ -7987,7 +8041,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>4611.62</v>
+        <v>4601.62</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -11653,13 +11707,13 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>5602.41</v>
+        <v>5597.41</v>
       </c>
       <c r="D175" t="n">
         <v>995.79</v>
       </c>
       <c r="E175" t="n">
-        <v>4606.62</v>
+        <v>4601.62</v>
       </c>
     </row>
     <row r="176">
@@ -11674,13 +11728,13 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>5102.41</v>
+        <v>5097.41</v>
       </c>
       <c r="D176" t="n">
         <v>495.79</v>
       </c>
       <c r="E176" t="n">
-        <v>4606.62</v>
+        <v>4601.62</v>
       </c>
     </row>
     <row r="177">
@@ -11695,13 +11749,13 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>4959.41</v>
+        <v>4954.41</v>
       </c>
       <c r="D177" t="n">
         <v>352.79</v>
       </c>
       <c r="E177" t="n">
-        <v>4606.62</v>
+        <v>4601.62</v>
       </c>
     </row>
     <row r="178">
@@ -11716,13 +11770,13 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>4733.41</v>
+        <v>4728.41</v>
       </c>
       <c r="D178" t="n">
         <v>126.79</v>
       </c>
       <c r="E178" t="n">
-        <v>4606.62</v>
+        <v>4601.62</v>
       </c>
     </row>
     <row r="179">
@@ -11737,13 +11791,13 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4607.41</v>
+        <v>4602.41</v>
       </c>
       <c r="D179" t="n">
         <v>0.79</v>
       </c>
       <c r="E179" t="n">
-        <v>4606.62</v>
+        <v>4601.62</v>
       </c>
     </row>
     <row r="180">
@@ -11758,13 +11812,13 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>20087.41</v>
+        <v>20077.41</v>
       </c>
       <c r="D180" t="n">
         <v>15475.79</v>
       </c>
       <c r="E180" t="n">
-        <v>4611.62</v>
+        <v>4601.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update 2026-10-02 12:11 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/57cfe36beb_Financial_Analysis_2026.xlsx
+++ b/57cfe36beb_Financial_Analysis_2026.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:G214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>كشف معاملات البطاقة 3390 (28/01/2026 - 01/10/2026)</t>
+          <t>كشف معاملات البطاقة 3390 (28/01/2026 - 02/10/2026)</t>
         </is>
       </c>
     </row>
@@ -6560,6 +6560,35 @@
       </c>
       <c r="G213" s="5" t="n">
         <v>20077.41</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>مصروف</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>talabat.com postpaid Maa</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>مطاعم وتوصيل</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="n">
+        <v>1372.26</v>
+      </c>
+      <c r="F214" s="5" t="n">
+        <v>14103.53</v>
+      </c>
+      <c r="G214" s="5" t="n">
+        <v>18705.15</v>
       </c>
     </row>
   </sheetData>
@@ -6861,22 +6890,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>2000</v>
+        <v>3372.26</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2000</v>
+        <v>3372.26</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>17000</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>15000</v>
+        <v>13627.74</v>
       </c>
     </row>
     <row r="14">
@@ -6886,22 +6915,22 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>101391.53</v>
+        <v>102763.79</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>9000</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>92391.53</v>
+        <v>93763.78999999999</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111725</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>19333.47</v>
+        <v>17961.21000000001</v>
       </c>
     </row>
   </sheetData>
@@ -6966,7 +6995,7 @@
         <v>39500</v>
       </c>
       <c r="D4" t="n">
-        <v>42.8</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="5">
@@ -6982,7 +7011,7 @@
         <v>14520</v>
       </c>
       <c r="D5" t="n">
-        <v>15.7</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="6">
@@ -6998,7 +7027,7 @@
         <v>13477.9</v>
       </c>
       <c r="D6" t="n">
-        <v>14.6</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="7">
@@ -7014,7 +7043,7 @@
         <v>8739.620000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>9.5</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -7024,13 +7053,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>5750.549999999999</v>
+        <v>7122.809999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>6.2</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="9">
@@ -7046,7 +7075,7 @@
         <v>3199.98</v>
       </c>
       <c r="D9" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="10">
@@ -7541,20 +7570,20 @@
         <v>17</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>46182</v>
+        <v>46297</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KASHIER*AboSh Cai</t>
+          <t>talabat.com postpaid Maa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>مشتريات ومحلات</t>
+          <t>مطاعم وتوصيل</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1350</v>
+        <v>1372.26</v>
       </c>
     </row>
     <row r="21">
@@ -7562,20 +7591,20 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>46235</v>
+        <v>46182</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>U TURN GI</t>
+          <t>KASHIER*AboSh Cai</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>أخرى (غير مصنف)</t>
+          <t>مشتريات ومحلات</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1150</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="22">
@@ -7583,20 +7612,20 @@
         <v>19</v>
       </c>
       <c r="B22" s="9" t="n">
-        <v>46156</v>
+        <v>46235</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EL EZABY HEL</t>
+          <t>U TURN GI</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>صحة وصيدليات</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1109.4</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="23">
@@ -7604,20 +7633,20 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>46266</v>
+        <v>46156</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BDC HARAM H</t>
+          <t>EL EZABY HEL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>صحة وصيدليات</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1100</v>
+        <v>1109.4</v>
       </c>
     </row>
   </sheetData>
@@ -7825,7 +7854,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>مؤشرات عامة - فترة 28/01/2026 حتى 01/10/2026</t>
+          <t>مؤشرات عامة - فترة 28/01/2026 حتى 02/10/2026</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7882,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
@@ -7864,7 +7893,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
@@ -7905,7 +7934,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>101391.53</v>
+        <v>102763.79</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -7927,7 +7956,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>92391.53</v>
+        <v>93763.78999999999</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
@@ -7953,7 +7982,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>52891.53</v>
+        <v>54263.79</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
@@ -7975,7 +8004,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>19333.47</v>
+        <v>17961.21</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
@@ -7986,7 +8015,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>374.05</v>
+        <v>378.08</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
@@ -7997,7 +8026,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>11386.23</v>
+        <v>11508.75</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
@@ -8019,7 +8048,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>20077.41</v>
+        <v>18705.15</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
@@ -8030,7 +8059,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>15475.79</v>
+        <v>14103.53</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
@@ -8060,7 +8089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11821,6 +11850,27 @@
         <v>4601.62</v>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>talabat.com postpaid Maa</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>18705.15</v>
+      </c>
+      <c r="D181" t="n">
+        <v>14103.53</v>
+      </c>
+      <c r="E181" t="n">
+        <v>4601.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>